<commit_message>
chore: refresh PWA precache (sw.js); update RBC sample workbook
- Regenerated Workbox precache after frontend build
- tsbuildinfo left unstaged (local TS incremental cache)

Made-with: Cursor
</commit_message>
<xml_diff>
--- a/Samples/RBC Georgia/RBC US STATEMENT 2025.xlsx
+++ b/Samples/RBC Georgia/RBC US STATEMENT 2025.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ozanbektas/Downloads/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ozanbektas/Documents/Business/Backtas Softwares/BCKTS_TECH/QuickYel/Samples/RBC Georgia/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{949BFDC6-99E8-6949-A3DD-A5833DE3252D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{61C640AC-4224-B44D-B20C-5DFEE1ABFC2E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18980" xr2:uid="{DB11FD69-CD5E-4360-9042-3A32A3847973}"/>
   </bookViews>
@@ -8374,7 +8374,6 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J1" xr:uid="{2DCD443B-B03F-4791-B8E0-98A6A00C56DB}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>